<commit_message>
login chưa chỉnh xong mới kết nối login
</commit_message>
<xml_diff>
--- a/test/appium_tests/result/result.xlsx
+++ b/test/appium_tests/result/result.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -768,6 +768,1125 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Lỗi: Message: Không tìm thấy thanh tìm kiếm cho query: Đánh đổi
+Stacktrace:
+NoSuchElementError: An element could not be located on the page using the given search parameters.
+    at AndroidUiautomator2Driver.findElOrEls (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-android-driver\lib\commands\find.js:75:11)
+    at processTicksAndRejections (internal/process/task_queues.js:97:5)
+    at AndroidUiautomator2Driver.findElOrElsWithProcessing (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:33:12)
+    at AndroidUiautomator2Driver.findElement (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:53:10)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2025-04-21 19:53:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Lỗi: Message: Không tìm thấy thanh tìm kiếm cho query: Đánh đổi
+Stacktrace:
+NoSuchElementError: An element could not be located on the page using the given search parameters.
+    at AndroidUiautomator2Driver.findElOrEls (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-android-driver\lib\commands\find.js:75:11)
+    at processTicksAndRejections (internal/process/task_queues.js:97:5)
+    at AndroidUiautomator2Driver.findElOrElsWithProcessing (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:33:12)
+    at AndroidUiautomator2Driver.findElement (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:53:10)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2025-04-21 19:59:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Lỗi: Message: Không tìm thấy thanh tìm kiếm cho query: Đánh đổi
+Stacktrace:
+NoSuchElementError: An element could not be located on the page using the given search parameters.
+    at AndroidUiautomator2Driver.findElOrEls (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-android-driver\lib\commands\find.js:75:11)
+    at runMicrotasks (&lt;anonymous&gt;)
+    at processTicksAndRejections (internal/process/task_queues.js:97:5)
+    at AndroidUiautomator2Driver.findElOrElsWithProcessing (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:33:12)
+    at AndroidUiautomator2Driver.findElement (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:53:10)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025-04-21 20:02:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Lỗi: Message: Không tìm thấy thanh tìm kiếm cho query: Đánh đổi
+Stacktrace:
+NoSuchElementError: An element could not be located on the page using the given search parameters.
+    at AndroidUiautomator2Driver.findElOrEls (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-android-driver\lib\commands\find.js:75:11)
+    at processTicksAndRejections (internal/process/task_queues.js:97:5)
+    at AndroidUiautomator2Driver.findElOrElsWithProcessing (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:33:12)
+    at AndroidUiautomator2Driver.findElement (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:53:10)</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2025-04-21 20:03:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Lỗi: Message: Không tìm thấy thanh tìm kiếm cho query: Đánh đổi
+Stacktrace:
+NoSuchElementError: An element could not be located on the page using the given search parameters.
+    at AndroidUiautomator2Driver.findElOrEls (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-android-driver\lib\commands\find.js:75:11)
+    at runMicrotasks (&lt;anonymous&gt;)
+    at processTicksAndRejections (internal/process/task_queues.js:97:5)
+    at AndroidUiautomator2Driver.findElOrElsWithProcessing (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:33:12)
+    at AndroidUiautomator2Driver.findElement (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:53:10)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2025-04-21 20:11:26</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Lỗi: Message: Không tìm thấy thanh tìm kiếm cho query: Đánh đổi
+Stacktrace:
+NoSuchElementError: An element could not be located on the page using the given search parameters.
+    at AndroidUiautomator2Driver.findElOrEls (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-android-driver\lib\commands\find.js:75:11)
+    at runMicrotasks (&lt;anonymous&gt;)
+    at processTicksAndRejections (internal/process/task_queues.js:97:5)
+    at AndroidUiautomator2Driver.findElOrElsWithProcessing (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:33:12)
+    at AndroidUiautomator2Driver.findElement (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:53:10)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2025-04-21 21:37:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Search Tab</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Lỗi khi chuyển sang tab Search: Message: Không tìm thấy tab Search
+Stacktrace:
+NoSuchElementError: An element could not be located on the page using the given search parameters.
+    at AndroidUiautomator2Driver.findElOrEls (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-android-driver\lib\commands\find.js:75:11)
+    at runMicrotasks (&lt;anonymous&gt;)
+    at processTicksAndRejections (internal/process/task_queues.js:97:5)
+    at AndroidUiautomator2Driver.findElOrElsWithProcessing (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:33:12)
+    at AndroidUiautomator2Driver.findElement (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:53:10)</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:04:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả cho 'Đánh đổi'</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:09:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả cho 'Fly me to the moon'</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:10:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả cho 'Obito'</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:10:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Không tìm thấy tiêu đề Search Results hoặc kết quả cho 'Đánh đổi'</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:18:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Không tìm thấy tiêu đề Search Results hoặc kết quả cho 'Fly me to the moon'</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:18:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Không tìm thấy tiêu đề Search Results hoặc kết quả cho 'Obito'</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:19:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Search Tab</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Lỗi khi chuyển sang tab Search: Message: Không tìm thấy tab Search
+Stacktrace:
+NoSuchElementError: An element could not be located on the page using the given search parameters.
+    at AndroidUiautomator2Driver.findElOrEls (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-android-driver\lib\commands\find.js:75:11)
+    at runMicrotasks (&lt;anonymous&gt;)
+    at processTicksAndRejections (internal/process/task_queues.js:97:5)
+    at AndroidUiautomator2Driver.findElOrElsWithProcessing (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:33:12)
+    at AndroidUiautomator2Driver.findElement (C:\Users\ADMIN\AppData\Local\Programs\Appium Server GUI\resources\app\node_modules\appium\node_modules\appium-base-driver\lib\basedriver\commands\find.js:53:10)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:25:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Không tìm thấy tiêu đề Search Results hoặc kết quả cho 'Đánh đổi'</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:32:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Không tìm thấy tiêu đề Search Results hoặc kết quả cho 'Fly me to the moon'</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:32:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Sequential Search</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Không tìm thấy tiêu đề Search Results hoặc kết quả cho 'Obito'</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:32:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Search Đánh đổi</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:42:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Search Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:42:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Search Obito</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:42:31</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Search Đánh đổi</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Không tìm thấy SongCard nào cho 'Đánh đổi'</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:55:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Search Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Không tìm thấy SongCard nào cho 'Fly me to the moon'</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:55:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Search Obito</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Không tìm thấy SongCard nào cho 'Obito'</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2025-04-21 22:55:30</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Search Đánh đổi</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Không tìm thấy SongCard nào cho 'Đánh đổi'</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2025-04-21 23:10:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Search Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Không tìm thấy SongCard nào cho 'Fly me to the moon'</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2025-04-21 23:10:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Search Obito</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>No results found</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2025-04-21 23:11:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Search Đánh đổi</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Không tìm thấy SongCard nào cho 'Đánh đổi'</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2025-04-21 23:20:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Search Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Không tìm thấy SongCard nào cho 'Fly me to the moon'</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2025-04-21 23:20:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Search Obito</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>No results found</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2025-04-21 23:20:56</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Search Đánh đổi</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả hoặc trạng thái 'No results found' cho 'Đánh đổi'</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2025-04-21 23:56:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Search Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả hoặc trạng thái 'No results found' cho 'Fly me to the moon'</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2025-04-21 23:57:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Search Obito</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả hoặc trạng thái 'No results found' cho 'Obito'</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2025-04-21 23:58:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Search Đánh đổi</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả hoặc trạng thái 'No results found' cho 'Đánh đổi'</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2025-04-22 00:21:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Search Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả hoặc trạng thái 'No results found' cho 'Fly me to the moon'</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2025-04-22 00:23:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Search Obito</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả hoặc trạng thái 'No results found' cho 'Obito'</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2025-04-22 00:24:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Search Đánh đổi</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Đánh đổi</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lỗi khi kiểm tra kết quả: Message: The element 'By.xpath: //android.widget.EditText[1]' is not linked to the same object in DOM anymore; For documentation on this error, please visit: https://www.selenium.dev/documentation/webdriver/troubleshooting/errors#stale-element-reference-exception
+Stacktrace:
+io.appium.uiautomator2.common.exceptions.StaleElementReferenceException: The element 'By.xpath: //android.widget.EditText[1]' is not linked to the same object in DOM anymore
+	at io.appium.uiautomator2.model.ElementsCache.restore(ElementsCache.java:122)
+	at io.appium.uiautomator2.model.ElementsCache.get(ElementsCache.java:153)
+	at io.appium.uiautomator2.handler.GetElementAttribute.safeHandle(GetElementAttribute.java:23)
+	at io.appium.uiautomator2.handler.request.SafeRequestHandler.handle(SafeRequestHandler.java:59)
+	at io.appium.uiautomator2.server.AppiumServlet.handleRequest(AppiumServlet.java:266)
+	at io.appium.uiautomator2.server.AppiumServlet.handleHttpRequest(AppiumServlet.java:260)
+	at io.appium.uiautomator2.http.ServerHandler.channelRead(ServerHandler.java:68)
+	at io.netty.channel.AbstractChannelHandlerContext.invokeChannelRead(AbstractChannelHandlerContext.java:366)
+	at io.netty.channel.AbstractChannelHandlerContext.invokeChannelRead(AbstractChannelHandlerContext.java:352)
+	at io.netty.channel.AbstractChannelHandlerContext.fireChannelRead(AbstractChannelHandlerContext.java:345)
+	at io.netty.handler.codec.MessageToMessageDecoder.channelRead(MessageToMessageDecoder.java:102)
+	at io.netty.channel.AbstractChannelHandlerContext.invokeChannelRead(AbstractChannelHandlerContext.java:366)
+	at io.netty.channel.AbstractChannelHandlerContext.invokeChannelRead(AbstractChannelHandlerContext.java:352)
+	at io.netty.channel.AbstractChannelHandlerContext.fireChannelRead(AbstractChannelHandlerContext.java:345)
+	at io.netty.channel.CombinedChannelDuplexHandler$DelegatingChannelHandlerContext.fireChannelRead(CombinedChannelDuplexHandler.java:435)
+	at io.netty.handler.codec.ByteToMessageDecoder.fireChannelRead(ByteToMessageDecoder.java:293)
+	at io.netty.handler.codec.ByteToMessageDecoder.channelRead(ByteToMessageDecoder.java:267)
+	at io.netty.channel.CombinedChannelDuplexHandler.channelRead(CombinedChannelDuplexHandler.java:250)
+	at io.netty.channel.AbstractChannelHandlerContext.invokeChannelRead(AbstractChannelHandlerContext.java:366)
+	at io.netty.channel.AbstractChannelHandlerContext.invokeChannelRead(AbstractChannelHandlerContext.java:352)
+	at io.netty.channel.AbstractChannelHandlerContext.fireChannelRead(AbstractChannelHandlerContext.java:345)
+	at io.netty.handler.timeout.IdleStateHandler.channelRead(IdleStateHandler.java:266)
+	at io.netty.channel.AbstractChannelHandlerContext.invokeChannelRead(AbstractChannelHandlerContext.java:366)
+	at io.netty.channel.AbstractChannelHandlerContext.invokeChannelRead(AbstractChannelHandlerContext.java:352)
+	at io.netty.channel.AbstractChannelHandlerContext.fireChannelRead(AbstractChannelHandlerContext.java:345)
+	at io.netty.channel.DefaultChannelPipeline$HeadContext.channelRead(DefaultChannelPipeline.java:1294)
+	at io.netty.channel.AbstractChannelHandlerContext.invokeChannelRead(AbstractChannelHandlerContext.java:366)
+	at io.netty.channel.AbstractChannelHandlerContext.invokeChannelRead(AbstractChannelHandlerContext.java:352)
+	at io.netty.channel.DefaultChannelPipeline.fireChannelRead(DefaultChannelPipeline.java:911)
+	at io.netty.channel.nio.AbstractNioByteChannel$NioByteUnsafe.read(AbstractNioByteChannel.java:131)
+	at io.netty.channel.nio.NioEventLoop.processSelectedKey(NioEventLoop.java:611)
+	at io.netty.channel.nio.NioEventLoop.processSelectedKeysOptimized(NioEventLoop.java:552)
+	at io.netty.channel.nio.NioEventLoop.processSelectedKeys(NioEventLoop.java:466)
+	at io.netty.channel.nio.NioEventLoop.run(NioEventLoop.java:438)
+	at io.netty.util.concurrent.SingleThreadEventExecutor$2.run(SingleThreadEventExecutor.java:140)
+	at io.netty.util.concurrent.DefaultThreadFactory$DefaultRunnableDecorator.run(DefaultThreadFactory.java:144)
+	at java.lang.Thread.run(Thread.java:1012)
+</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2025-04-22 00:37:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Search Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Fly me to the moon</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả hoặc trạng thái 'No results found' cho 'Fly me to the moon'</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2025-04-22 00:39:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Search Obito</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Obito</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Không tìm thấy kết quả hoặc trạng thái 'No results found' cho 'Obito'</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2025-04-22 00:41:09</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>